<commit_message>
Add 2026 school project total cost to hakediş workbook
Include III.B ortaokul unit cost × gross area summary and kalıp
share versus overall project approximate price.

Co-authored-by: barsokrr <barsokrr@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/metraj/Kalip_Hakedis_Tablosu.xlsx
+++ b/metraj/Kalip_Hakedis_Tablosu.xlsx
@@ -7,11 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="HAKEDIS ICMAL" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="TEK HAKEDIS CETVELI" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="DONEM DETAY" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ALTERNATIF FIYAT" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="IMZA" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="OKUL TOPLAM FIYAT" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="HAKEDIS ICMAL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="TEK HAKEDIS CETVELI" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="DONEM DETAY" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ALTERNATIF FIYAT" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="IMZA" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,6 +75,28 @@
     <font>
       <b val="1"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00006600"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="7">
@@ -155,7 +178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -198,6 +221,13 @@
     <xf numFmtId="4" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="11" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="12" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -563,6 +593,575 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>KARŞIYAKA ORTAOKULU (24 DERSLİK) — PROJE TOPLAM YAKLAŞIK FİYAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Dayanak: 2026 Yapı Yaklaşık Birim Maliyetleri Tebliği (RG 03.02.2026 / 33157) | KDV hariç, GG %15 + kâr %10 dahil</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>A) YAPI SINIFI</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="34" t="inlineStr">
+        <is>
+          <t>Kalem</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>Değer</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Proje</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Karşıyaka Ortaokulu (24 derslik)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Yapı sınıfı (ana)</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>III. Sınıf (B) Grubu</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Tanım</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>İlkokul ve ortaokul yapıları</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>2026 birim maliyet (BM)</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>21.050,00 TL/m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Alternatif (spor/konferanslı büyük okul)</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>IV,B — 33.900,00 TL/m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>B) İNŞAAT ALANI</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="34" t="inlineStr">
+        <is>
+          <t>Kalem</t>
+        </is>
+      </c>
+      <c r="B14" s="34" t="inlineStr">
+        <is>
+          <t>Hesap</t>
+        </is>
+      </c>
+      <c r="C14" s="34" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Tipik kat</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>51,18 × 20,09</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="n">
+        <v>1028.21</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>5 kat (döşemeler)</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>kat × 5</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="n">
+        <v>5141.03</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="28" t="inlineStr">
+        <is>
+          <t>6 kat (bodrum+5) — ana hesap</t>
+        </is>
+      </c>
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>kat × 6</t>
+        </is>
+      </c>
+      <c r="C17" s="33" t="n">
+        <v>6169.24</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>C) OKUL PROJESİ TOPLAM YAKLAŞIK FİYAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="35" t="inlineStr">
+        <is>
+          <t>Senaryo</t>
+        </is>
+      </c>
+      <c r="B21" s="35" t="inlineStr">
+        <is>
+          <t>Alan m²</t>
+        </is>
+      </c>
+      <c r="C21" s="35" t="inlineStr">
+        <is>
+          <t>BM TL/m²</t>
+        </is>
+      </c>
+      <c r="D21" s="35" t="inlineStr">
+        <is>
+          <t>Toplam (KDV hariç) TL</t>
+        </is>
+      </c>
+      <c r="E21" s="35" t="inlineStr">
+        <is>
+          <t>KDV %20 TL</t>
+        </is>
+      </c>
+      <c r="F21" s="35" t="inlineStr">
+        <is>
+          <t>KDV Dahil TL</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Ana — Ortaokul III.B × 6 kat</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="n">
+        <v>6169.24</v>
+      </c>
+      <c r="C22" s="19" t="n">
+        <v>21050</v>
+      </c>
+      <c r="D22" s="19" t="n">
+        <v>129862443.06</v>
+      </c>
+      <c r="E22" s="19" t="n">
+        <v>25972488.61</v>
+      </c>
+      <c r="F22" s="19" t="n">
+        <v>155834931.67</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Ortaokul III.B × 5 kat</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="n">
+        <v>5141.03</v>
+      </c>
+      <c r="C23" s="17" t="n">
+        <v>21050</v>
+      </c>
+      <c r="D23" s="17" t="n">
+        <v>108218702.55</v>
+      </c>
+      <c r="E23" s="17" t="n">
+        <v>21643740.51</v>
+      </c>
+      <c r="F23" s="17" t="n">
+        <v>129862443.06</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Büyük okul IV.B × 6 kat (alternatif)</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="n">
+        <v>6169.24</v>
+      </c>
+      <c r="C24" s="17" t="n">
+        <v>33900</v>
+      </c>
+      <c r="D24" s="17" t="n">
+        <v>209137141.08</v>
+      </c>
+      <c r="E24" s="17" t="n">
+        <v>41827428.22</v>
+      </c>
+      <c r="F24" s="17" t="n">
+        <v>250964569.3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="26" t="inlineStr">
+        <is>
+          <t>OKUL PROJESİ TOPLAM FİYAT (ANA)</t>
+        </is>
+      </c>
+      <c r="B26" s="36" t="n">
+        <v>129862443.06</v>
+      </c>
+      <c r="C26" s="26" t="inlineStr">
+        <is>
+          <t>TL (KDV hariç)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>KDV dahil genel toplam</t>
+        </is>
+      </c>
+      <c r="B27" s="37" t="n">
+        <v>155834931.67</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Hesap: 6.169,24 m² × 21.050,00 TL/m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>D) KALIP İŞÇİLİĞİNİN PROJE İÇİNDEKİ PAYI</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="34" t="inlineStr">
+        <is>
+          <t>Kalem</t>
+        </is>
+      </c>
+      <c r="B31" s="34" t="inlineStr">
+        <is>
+          <t>Tutar TL</t>
+        </is>
+      </c>
+      <c r="C31" s="34" t="inlineStr">
+        <is>
+          <t>Oran</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Okul toplam (KDV hariç)</t>
+        </is>
+      </c>
+      <c r="B32" s="17" t="n">
+        <v>129862443.06</v>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Kalıp işçiliği 11.773 m² × 470 (KDV hariç)</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="n">
+        <v>5533498</v>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>4.26%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Kalıp işçiliği (KDV dahil)</t>
+        </is>
+      </c>
+      <c r="B34" s="17" t="n">
+        <v>6640197.6</v>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>4.26%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Kalıp dışı diğer işler (KDV hariç, yaklaşık)</t>
+        </is>
+      </c>
+      <c r="B35" s="17" t="n">
+        <v>124328945.06</v>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>95.74%</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>E) TEK BAKIŞTA ÖZET</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="34" t="inlineStr">
+        <is>
+          <t>Kalem</t>
+        </is>
+      </c>
+      <c r="B39" s="34" t="inlineStr">
+        <is>
+          <t>Değer</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>Okul tipi</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>24 derslik ortaokul</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>Yapı sınıfı</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>III.B — İlkokul/ortaokul</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>Brüt inşaat alanı</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>6.169,2 m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>2026 BM</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>21.050 TL/m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="18" t="inlineStr">
+        <is>
+          <t>OKUL TOPLAM (KDV hariç)</t>
+        </is>
+      </c>
+      <c r="B44" s="18" t="inlineStr">
+        <is>
+          <t>129.862.443 TL</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="18" t="inlineStr">
+        <is>
+          <t>OKUL TOPLAM (KDV dahil)</t>
+        </is>
+      </c>
+      <c r="B45" s="18" t="inlineStr">
+        <is>
+          <t>155.834.932 TL</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>Kalıp işçiliği (KDV hariç)</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>5.533.498 TL</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>Kalıp / proje oranı</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>%4.26</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="20" t="inlineStr">
+        <is>
+          <t>NOTLAR:</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="20" t="inlineStr">
+        <is>
+          <t>• Toplam fiyat; arsa, çevre düzenlemesi ve bina dışı altyapıyı içermez (tebliğ hükmü).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="20" t="inlineStr">
+        <is>
+          <t>• Birim maliyet mimarlık-mühendislik hizmet bedeli hesabı içindir; ihale keşfi yerine geçmez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="20" t="inlineStr">
+        <is>
+          <t>• Ana senaryo: III.B ortaokul × 6 kat brüt alan. Spor salonu/konferans salonu varsa IV.B (33.900 TL/m²) değerlendirilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="20" t="inlineStr">
+        <is>
+          <t>• Kalıp tutarı yalnız işçiliktir (470 TL/m²); proje toplamının içindeki pay yaklaşık gösterimdir.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="A52:F52"/>
+    <mergeCell ref="A54:F54"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="A53:F53"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:O36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -611,6 +1210,13 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="38" t="inlineStr">
+        <is>
+          <t>OKUL PROJE TOPLAM YAKLAŞIK FİYAT (III.B × 6,169 m² × 21,050 TL/m²): 129,862,443 TL KDV hariç / 155,834,932 TL KDV dahil | Detay: OKUL TOPLAM FIYAT sayfası</t>
+        </is>
+      </c>
+    </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -1421,13 +2027,14 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A35:H35"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A5:L5"/>
     <mergeCell ref="A32:H32"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="A33:H33"/>
@@ -1442,7 +2049,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1471,7 +2078,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Karşıyaka Ortaokulu | Kalıp işçiliği | Birim fiyat 470 TL/m² | Kırık ölçü</t>
+          <t>Karşıyaka Ortaokulu | Kalıp işçiliği 470 TL/m² | Okul toplam ≈ 129.9 M TL (KDV hariç, III.B)</t>
         </is>
       </c>
     </row>
@@ -1861,7 +2468,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3045,16 +3652,16 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A36:H36"/>
     <mergeCell ref="A25:H25"/>
     <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A36:H36"/>
     <mergeCell ref="A14:H14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3253,7 +3860,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>